<commit_message>
Add DMEM as storage medium for sample metadata
Closes #184
</commit_message>
<xml_diff>
--- a/sample-block/latest/sample-block.xlsx
+++ b/sample-block/latest/sample-block.xlsx
@@ -42,10 +42,10 @@
     </comment>
     <comment ref="C1" authorId="1">
       <text>
-        <t>A locally assigned identifier provided by the data provider for the dataset. It
-is used to reference an external metadata record that may be maintained
-independently, enabling traceability and supporting provenance tracking.
-Example: Visium_9OLC_A4_S1</t>
+        <t>An identifier assigned by the data provider to reference an external metadata
+record for the dataset. The external record may be maintained independently and
+can support dataset traceability and provenance tracking. Leave this field empty
+if no such identifier exists.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="1">
@@ -188,7 +188,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="179">
   <si>
     <t>source_id</t>
   </si>
@@ -208,12 +208,24 @@
     <t>source_storage_duration_unit</t>
   </si>
   <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
+  </si>
+  <si>
     <t>hour</t>
   </si>
   <si>
     <t>http://purl.obolibrary.org/obo/UO_0000032</t>
   </si>
   <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
+  </si>
+  <si>
     <t>month</t>
   </si>
   <si>
@@ -226,48 +238,36 @@
     <t>http://purl.obolibrary.org/obo/UO_0000036</t>
   </si>
   <si>
-    <t>day</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
-  </si>
-  <si>
-    <t>minute</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
-  </si>
-  <si>
     <t>tissue_weight_value</t>
   </si>
   <si>
     <t>tissue_weight_unit</t>
   </si>
   <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000009</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000021</t>
+  </si>
+  <si>
+    <t>mg</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000022</t>
+  </si>
+  <si>
     <t>ug</t>
   </si>
   <si>
     <t>http://purl.obolibrary.org/obo/UO_0000023</t>
   </si>
   <si>
-    <t>g</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000021</t>
-  </si>
-  <si>
-    <t>mg</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000022</t>
-  </si>
-  <si>
-    <t>kg</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000009</t>
-  </si>
-  <si>
     <t>volume_value</t>
   </si>
   <si>
@@ -280,67 +280,211 @@
     <t>http://purl.obolibrary.org/obo/UO_0000097</t>
   </si>
   <si>
+    <t>ml</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000098</t>
+  </si>
+  <si>
+    <t>um^3</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000112</t>
+  </si>
+  <si>
     <t>mm^3</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000136</t>
   </si>
   <si>
-    <t>um^3</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000112</t>
-  </si>
-  <si>
-    <t>ml</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000098</t>
-  </si>
-  <si>
     <t>pathology_distance_value</t>
   </si>
   <si>
     <t>pathology_distance_unit</t>
   </si>
   <si>
+    <t>cm</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000015</t>
+  </si>
+  <si>
     <t>mm</t>
   </si>
   <si>
     <t>http://purl.obolibrary.org/obo/UO_0000016</t>
   </si>
   <si>
-    <t>cm</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000015</t>
-  </si>
-  <si>
     <t>preparation_medium</t>
   </si>
   <si>
+    <t>Lysis buffer</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C178573</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
+  </si>
+  <si>
+    <t>PAXgene tissue kit (PXT)</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185113</t>
+  </si>
+  <si>
+    <t>DMEM</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185409</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C41132</t>
+  </si>
+  <si>
+    <t>RNAlater</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C63348</t>
+  </si>
+  <si>
+    <t>PLP (Periodate-Lysine-Paraformaldehyde)</t>
+  </si>
+  <si>
+    <t>http://purl.bioontology.org/ontology/MESH/C046311</t>
+  </si>
+  <si>
+    <t>Ethanol</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_16236</t>
+  </si>
+  <si>
+    <t>Methanol</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_17790</t>
+  </si>
+  <si>
+    <t>PFA (Paraformaldehyde)</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_61538</t>
+  </si>
+  <si>
+    <t>NBF (Neutral Buffered Formalin)</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/OBIB_0000213</t>
+  </si>
+  <si>
+    <t>PBS</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/OBI_0100046</t>
+  </si>
+  <si>
+    <t>MACS tissue storage solution</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000105</t>
+  </si>
+  <si>
+    <t>Inflated (Agarose)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000106</t>
+  </si>
+  <si>
+    <t>Fixed frozen OCT (Formalin, sucrose protected)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000116</t>
+  </si>
+  <si>
+    <t>Allprotect tissue reagent (ALL)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000118</t>
+  </si>
+  <si>
+    <t>Inflated (OCT)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000123</t>
+  </si>
+  <si>
+    <t>Fresh frozen OCT</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000126</t>
+  </si>
+  <si>
+    <t>Fresh frozen CMC</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000130</t>
+  </si>
+  <si>
+    <t>CLARITY hydrogel</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000134</t>
+  </si>
+  <si>
+    <t>Bouin's</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000140</t>
+  </si>
+  <si>
+    <t>Fixed frozen OCT (PFA, sucrose protected)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000147</t>
+  </si>
+  <si>
+    <t>Fixed frozen OCT (Cytofix/Cytoperm)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000149</t>
+  </si>
+  <si>
+    <t>UW Solution</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000151</t>
+  </si>
+  <si>
     <t>HTK Solution</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000152</t>
   </si>
   <si>
-    <t>NBF (Neutral Buffered Formalin)</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/OBIB_0000213</t>
-  </si>
-  <si>
-    <t>Allprotect tissue reagent (ALL)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000118</t>
-  </si>
-  <si>
-    <t>CLARITY hydrogel</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000134</t>
+    <t>Fresh frozen gelatin</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000198</t>
+  </si>
+  <si>
+    <t>Perfadex Plus</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000249</t>
+  </si>
+  <si>
+    <t>Biops buffer</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000330</t>
   </si>
   <si>
     <t>Trumps fixative</t>
@@ -349,229 +493,91 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000331</t>
   </si>
   <si>
+    <t>2% PFA/2.5% Glutaraldehyde</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000332</t>
+  </si>
+  <si>
+    <t>Modified Davidson's Fixative</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000370</t>
+  </si>
+  <si>
+    <t>Alpha-MEM</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000371</t>
+  </si>
+  <si>
+    <t>Growth media</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000372</t>
+  </si>
+  <si>
+    <t>HPMC-PVP</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000386</t>
+  </si>
+  <si>
     <t>1X fixation &amp; permeabilization buffer</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000425</t>
   </si>
   <si>
-    <t>Inflated (OCT)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000123</t>
-  </si>
-  <si>
-    <t>DMEM</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185409</t>
-  </si>
-  <si>
-    <t>Perfadex Plus</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000249</t>
-  </si>
-  <si>
-    <t>PFA (Paraformaldehyde)</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_61538</t>
-  </si>
-  <si>
-    <t>Fixed frozen OCT (Formalin, sucrose protected)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000116</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
-  </si>
-  <si>
-    <t>Fresh frozen OCT</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000126</t>
-  </si>
-  <si>
-    <t>Alpha-MEM</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000371</t>
-  </si>
-  <si>
-    <t>2% PFA/2.5% Glutaraldehyde</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000332</t>
-  </si>
-  <si>
-    <t>Bouin's</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000140</t>
-  </si>
-  <si>
-    <t>Methanol</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_17790</t>
-  </si>
-  <si>
-    <t>PAXgene tissue kit (PXT)</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185113</t>
-  </si>
-  <si>
-    <t>PBS</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/OBI_0100046</t>
-  </si>
-  <si>
-    <t>Ethanol</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_16236</t>
-  </si>
-  <si>
-    <t>Modified Davidson's Fixative</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000370</t>
-  </si>
-  <si>
-    <t>HPMC-PVP</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000386</t>
-  </si>
-  <si>
-    <t>Inflated (Agarose)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000106</t>
-  </si>
-  <si>
-    <t>PLP (Periodate-Lysine-Paraformaldehyde)</t>
-  </si>
-  <si>
-    <t>http://purl.bioontology.org/ontology/MESH/C046311</t>
-  </si>
-  <si>
-    <t>UW Solution</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000151</t>
-  </si>
-  <si>
-    <t>MACS tissue storage solution</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000105</t>
-  </si>
-  <si>
-    <t>Fresh frozen CMC</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000130</t>
-  </si>
-  <si>
-    <t>Fresh frozen gelatin</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000198</t>
-  </si>
-  <si>
-    <t>Growth media</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000372</t>
-  </si>
-  <si>
-    <t>RNAlater</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C63348</t>
-  </si>
-  <si>
-    <t>Biops buffer</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000330</t>
-  </si>
-  <si>
-    <t>Fixed frozen OCT (Cytofix/Cytoperm)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000149</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C41132</t>
-  </si>
-  <si>
-    <t>Fixed frozen OCT (PFA, sucrose protected)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000147</t>
-  </si>
-  <si>
-    <t>Lysis buffer</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C178573</t>
-  </si>
-  <si>
     <t>preparation_condition</t>
   </si>
   <si>
+    <t>Frozen in liquid nitrogen</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185338</t>
+  </si>
+  <si>
     <t>Frozen in liquid nitrogen vapor</t>
   </si>
   <si>
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185339</t>
   </si>
   <si>
+    <t>Frozen on dry ice</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C187069</t>
+  </si>
+  <si>
     <t>Stored in ambient temperature</t>
   </si>
   <si>
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C70719</t>
   </si>
   <si>
+    <t>Stored in refrigerator</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000104</t>
+  </si>
+  <si>
+    <t>Frozen at -20 degrees celsius</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000107</t>
+  </si>
+  <si>
     <t>Frozen on ice</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000144</t>
   </si>
   <si>
-    <t>Frozen in liquid nitrogen</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C185338</t>
-  </si>
-  <si>
-    <t>Frozen at -20 degrees celsius</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000107</t>
-  </si>
-  <si>
-    <t>Frozen on dry ice</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C187069</t>
-  </si>
-  <si>
-    <t>Stored in refrigerator</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000104</t>
+    <t>Incubated at 37 degrees celsius</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000148</t>
   </si>
   <si>
     <t>Stored on wet ice</t>
@@ -589,16 +595,40 @@
     <t>storage_medium</t>
   </si>
   <si>
+    <t>FFPE (Paraffin embedded)</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C143028</t>
+  </si>
+  <si>
+    <t>OCT</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C63523</t>
+  </si>
+  <si>
     <t>Water</t>
   </si>
   <si>
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65147</t>
   </si>
   <si>
-    <t>OCT</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C63523</t>
+    <t>Gelatin</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65802</t>
+  </si>
+  <si>
+    <t>CMC</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C83594</t>
+  </si>
+  <si>
+    <t>Formic acid in water</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C83719</t>
   </si>
   <si>
     <t>DMSO (no serum)</t>
@@ -607,22 +637,28 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000115</t>
   </si>
   <si>
-    <t>Gelatin</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65802</t>
-  </si>
-  <si>
     <t>DMSO (serum)</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000125</t>
   </si>
   <si>
-    <t>CMC</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C83594</t>
+    <t>Tris-EDTA</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000135</t>
+  </si>
+  <si>
+    <t>Cryo-EM</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000333</t>
+  </si>
+  <si>
+    <t>Concentrated quench buffer</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000391</t>
   </si>
   <si>
     <t>1X quench buffer</t>
@@ -631,57 +667,27 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000427</t>
   </si>
   <si>
-    <t>Formic acid in water</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C83719</t>
-  </si>
-  <si>
-    <t>Tris-EDTA</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000135</t>
-  </si>
-  <si>
-    <t>Concentrated quench buffer</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000391</t>
-  </si>
-  <si>
-    <t>Cryo-EM</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000333</t>
-  </si>
-  <si>
-    <t>FFPE (Paraffin embedded)</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C143028</t>
+    <t>Nuclease-free water</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000482</t>
   </si>
   <si>
     <t>storage_method</t>
   </si>
   <si>
+    <t>Frozen at -80 degrees celsius</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000132</t>
+  </si>
+  <si>
     <t>Stored in desiccator</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000387</t>
   </si>
   <si>
-    <t>Incubated at 37 degrees celsius</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000148</t>
-  </si>
-  <si>
-    <t>Frozen at -80 degrees celsius</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000132</t>
-  </si>
-  <si>
     <t>quality_criteria</t>
   </si>
   <si>
@@ -712,7 +718,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2025-11-03T17:31:46-08:00</t>
+    <t>2026-10-05T17:22:34-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -879,33 +885,33 @@
         <v>113</v>
       </c>
       <c r="O1" t="s" s="1">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="P1" t="s" s="1">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="Q1" t="s" s="1">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="R1" t="s" s="1">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="S1" t="s" s="1">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="T1" t="s" s="1">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="U1" t="s" s="1">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="V1" t="s" s="1">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2">
       <c r="V2" t="s" s="23">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -942,7 +948,7 @@
       <formula1>'preparation_medium'!$A$1:$A$35</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="N2:N1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_condition'!$A$1:$A$9</formula1>
+      <formula1>'preparation_condition'!$A$1:$A$10</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" sqref="O2:O1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be greater than 0" showErrorMessage="true">
       <formula1>0</formula1>
@@ -952,7 +958,7 @@
       <formula1>'processing_time_unit'!$A$1:$A$3</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="Q2:Q1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'storage_medium'!$A$1:$A$25</formula1>
+      <formula1>'storage_medium'!$A$1:$A$27</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="R2:R1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
       <formula1>'storage_method'!$A$1:$A$12</formula1>
@@ -971,98 +977,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>115</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>66</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>159</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>160</v>
+        <v>122</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>161</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>162</v>
+        <v>124</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>163</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>122</v>
+        <v>162</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>108</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -1083,30 +1089,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -1566,47 +1572,47 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>114</v>
+        <v>45</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>115</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>66</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6">
@@ -1639,6 +1645,14 @@
       </c>
       <c r="B9" t="s" s="0">
         <v>129</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -1661,18 +1675,18 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1682,63 +1696,63 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>135</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>136</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>137</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>138</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>65</v>
+        <v>137</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>66</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8">
@@ -1767,74 +1781,74 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>71</v>
+        <v>145</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>72</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>76</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>78</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>80</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>145</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>146</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>82</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>147</v>
+        <v>67</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>148</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>86</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>94</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20">
@@ -1855,34 +1869,50 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>153</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>154</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>101</v>
+        <v>153</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>102</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>155</v>
+        <v>109</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>156</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>107</v>
+        <v>155</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>108</v>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>